<commit_message>
Updated HvdP of fcVeghel added `"isFormerMember": true` to suppress "warning" crash on Debug builds.
</commit_message>
<xml_diff>
--- a/JSON/ClubsNL.xlsx
+++ b/JSON/ClubsNL.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10222"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/petervandenhamer/Developer/Xcode projects/SwiftUI/Photo-Club-Hub/JSON/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/petervandenhamer/Developer/Xcode projects/SwiftUI/Photo Club Hub/JSON/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{56737D37-1151-134A-B046-3B906C498E4B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38AD0530-B716-DB4C-8283-D4DAFFD147DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16660" xr2:uid="{084E1DFC-5E29-0141-8377-174496560C67}"/>
   </bookViews>
@@ -1743,10 +1743,10 @@
         <v>95</v>
       </c>
       <c r="C24" s="21">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="D24" s="13">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="E24" s="12" t="s">
         <v>18</v>
@@ -2327,11 +2327,11 @@
       </c>
       <c r="C39" s="9">
         <f>SUM(C23:C37)</f>
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="D39" s="9">
         <f>SUM(D23:D37)</f>
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="E39" s="14"/>
       <c r="F39" s="15"/>
@@ -2349,7 +2349,7 @@
       </c>
       <c r="C40" s="40">
         <f>1 - C39/D39</f>
-        <v>0.27459016393442626</v>
+        <v>0.27572016460905346</v>
       </c>
     </row>
     <row r="41" spans="1:14" ht="17" thickTop="1">

</xml_diff>

<commit_message>
Added extra member JK for fgOirschot
</commit_message>
<xml_diff>
--- a/JSON/ClubsNL.xlsx
+++ b/JSON/ClubsNL.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10322"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/petervandenhamer/Developer/Xcode projects/SwiftUI/Photo Club Hub/JSON/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{38AD0530-B716-DB4C-8283-D4DAFFD147DA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1CBB933-BA89-754C-8423-FDC7AABBEA21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16660" xr2:uid="{084E1DFC-5E29-0141-8377-174496560C67}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="51200" windowHeight="28800" xr2:uid="{084E1DFC-5E29-0141-8377-174496560C67}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -113,7 +113,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="97">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="98">
   <si>
     <t>Club</t>
   </si>
@@ -404,6 +404,9 @@
   </si>
   <si>
     <t>besproken/goedgekeurd op club ALV op 5-Feb-26</t>
+  </si>
+  <si>
+    <t>Anneke Hooijer?</t>
   </si>
 </sst>
 </file>
@@ -2473,7 +2476,7 @@
         <v>23</v>
       </c>
       <c r="B46" t="s">
-        <v>15</v>
+        <v>97</v>
       </c>
       <c r="C46" s="3">
         <v>10</v>

</xml_diff>

<commit_message>
Maintenance to data in ClubsNL.xlsx
</commit_message>
<xml_diff>
--- a/JSON/ClubsNL.xlsx
+++ b/JSON/ClubsNL.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/petervandenhamer/Developer/Xcode projects/SwiftUI/Photo Club Hub/JSON/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1CBB933-BA89-754C-8423-FDC7AABBEA21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{930166F2-91F6-F741-B553-8B9C7B9A0B88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="51200" windowHeight="28800" xr2:uid="{084E1DFC-5E29-0141-8377-174496560C67}"/>
+    <workbookView xWindow="5320" yWindow="760" windowWidth="29400" windowHeight="24720" xr2:uid="{084E1DFC-5E29-0141-8377-174496560C67}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -145,9 +145,6 @@
     <t>Paula Anglès</t>
   </si>
   <si>
-    <t>Wil der Kinderen</t>
-  </si>
-  <si>
     <t>Bob Alisic</t>
   </si>
   <si>
@@ -407,6 +404,9 @@
   </si>
   <si>
     <t>Anneke Hooijer?</t>
+  </si>
+  <si>
+    <t>Henk Verbeek</t>
   </si>
 </sst>
 </file>
@@ -1444,19 +1444,19 @@
   <sheetData>
     <row r="1" spans="1:7" s="1" customFormat="1">
       <c r="A1" s="1" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="G1" s="7"/>
     </row>
     <row r="3" spans="1:7" s="36" customFormat="1">
       <c r="B3" s="37" t="s">
+        <v>71</v>
+      </c>
+      <c r="C3" s="37" t="s">
+        <v>70</v>
+      </c>
+      <c r="D3" s="37" t="s">
         <v>72</v>
-      </c>
-      <c r="C3" s="37" t="s">
-        <v>71</v>
-      </c>
-      <c r="D3" s="37" t="s">
-        <v>73</v>
       </c>
       <c r="G3" s="42"/>
     </row>
@@ -1468,7 +1468,7 @@
         <v>0</v>
       </c>
       <c r="D4" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
     </row>
     <row r="5" spans="1:7">
@@ -1479,29 +1479,29 @@
         <v>0</v>
       </c>
       <c r="D5" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" spans="1:7">
       <c r="B6" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C6">
         <v>10</v>
       </c>
       <c r="D6" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="7" spans="1:7">
       <c r="B7" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C7">
         <v>79</v>
       </c>
       <c r="D7" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="8" spans="1:7">
@@ -1512,7 +1512,7 @@
         <v>2</v>
       </c>
       <c r="D8" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="9" spans="1:7">
@@ -1523,7 +1523,7 @@
         <v>13</v>
       </c>
       <c r="D9" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
     </row>
     <row r="10" spans="1:7">
@@ -1534,7 +1534,7 @@
         <v>3</v>
       </c>
       <c r="D10" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
     </row>
     <row r="11" spans="1:7">
@@ -1545,7 +1545,7 @@
         <v>3</v>
       </c>
       <c r="D11" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
     </row>
     <row r="12" spans="1:7">
@@ -1556,7 +1556,7 @@
         <v>2</v>
       </c>
       <c r="D12" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="13" spans="1:7">
@@ -1567,7 +1567,7 @@
         <v>2</v>
       </c>
       <c r="D13" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="14" spans="1:7">
@@ -1578,7 +1578,7 @@
         <v>2</v>
       </c>
       <c r="D14" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="15" spans="1:7">
@@ -1589,7 +1589,7 @@
         <v>10</v>
       </c>
       <c r="D15" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="16" spans="1:7">
@@ -1600,12 +1600,12 @@
         <v>6</v>
       </c>
       <c r="D16" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="18" spans="1:17">
       <c r="B18" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C18">
         <f>SUM(C4:C17)</f>
@@ -1614,7 +1614,7 @@
     </row>
     <row r="19" spans="1:17">
       <c r="B19" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C19">
         <f>SUM(C5:C8)-C8</f>
@@ -1626,22 +1626,22 @@
       <c r="A21"/>
       <c r="B21"/>
       <c r="C21" s="50" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="D21" s="48"/>
       <c r="E21" s="47" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F21" s="48"/>
       <c r="G21" s="47" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="H21" s="49"/>
       <c r="I21" s="49"/>
       <c r="J21" s="49"/>
       <c r="K21" s="48"/>
       <c r="L21" s="38" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="M21"/>
       <c r="N21"/>
@@ -1654,43 +1654,43 @@
         <v>0</v>
       </c>
       <c r="B22" s="6" t="s">
+        <v>61</v>
+      </c>
+      <c r="C22" s="20" t="s">
         <v>62</v>
       </c>
-      <c r="C22" s="20" t="s">
+      <c r="D22" s="11" t="s">
         <v>63</v>
       </c>
-      <c r="D22" s="11" t="s">
-        <v>64</v>
-      </c>
       <c r="E22" s="10" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="F22" s="11" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="G22" s="10" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="H22" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="I22" s="17" t="s">
+        <v>26</v>
+      </c>
+      <c r="J22" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="K22" s="11" t="s">
+        <v>50</v>
+      </c>
+      <c r="L22" s="18" t="s">
+        <v>19</v>
+      </c>
+      <c r="M22" s="8" t="s">
+        <v>30</v>
+      </c>
+      <c r="N22" s="6" t="s">
         <v>29</v>
-      </c>
-      <c r="I22" s="17" t="s">
-        <v>27</v>
-      </c>
-      <c r="J22" s="17" t="s">
-        <v>53</v>
-      </c>
-      <c r="K22" s="11" t="s">
-        <v>51</v>
-      </c>
-      <c r="L22" s="18" t="s">
-        <v>20</v>
-      </c>
-      <c r="M22" s="8" t="s">
-        <v>31</v>
-      </c>
-      <c r="N22" s="6" t="s">
-        <v>30</v>
       </c>
       <c r="O22"/>
       <c r="P22"/>
@@ -1698,10 +1698,10 @@
     </row>
     <row r="23" spans="1:17" ht="20" customHeight="1">
       <c r="A23" s="4" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B23" s="4" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C23" s="22">
         <v>0</v>
@@ -1710,40 +1710,40 @@
         <v>35</v>
       </c>
       <c r="E23" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="F23" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="G23" s="41" t="s">
         <v>18</v>
       </c>
-      <c r="F23" s="25" t="s">
+      <c r="H23" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="G23" s="41" t="s">
-        <v>19</v>
-      </c>
-      <c r="H23" s="3" t="s">
-        <v>19</v>
-      </c>
       <c r="I23" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J23" s="26" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K23" s="25" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="L23" s="27" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="M23" s="5"/>
       <c r="N23" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
     </row>
     <row r="24" spans="1:17" ht="20" customHeight="1">
       <c r="A24" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B24" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C24" s="21">
         <v>34</v>
@@ -1752,34 +1752,34 @@
         <v>34</v>
       </c>
       <c r="E24" s="12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F24" s="13" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G24" s="43" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H24" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I24" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J24" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="K24" s="25" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L24" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="M24" s="26" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="N24" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="25" spans="1:17" ht="20" customHeight="1">
@@ -1796,28 +1796,28 @@
         <v>22</v>
       </c>
       <c r="E25" s="12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F25" s="25" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G25" s="41" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I25" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J25" s="3">
         <v>7</v>
       </c>
       <c r="K25" s="25" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L25" s="28" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M25" s="3"/>
     </row>
@@ -1835,34 +1835,34 @@
         <v>24</v>
       </c>
       <c r="E26" s="12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F26" s="13" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G26" s="41" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H26" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I26" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J26" s="3">
         <v>8</v>
       </c>
       <c r="K26" s="13" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L26" s="28" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M26" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="N26" s="30" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="27" spans="1:17" ht="20" customHeight="1">
@@ -1870,37 +1870,37 @@
         <v>5</v>
       </c>
       <c r="B27" t="s">
-        <v>10</v>
-      </c>
-      <c r="C27" s="24">
-        <v>18</v>
+        <v>97</v>
+      </c>
+      <c r="C27" s="21">
+        <v>19</v>
       </c>
       <c r="D27" s="13">
         <v>19</v>
       </c>
       <c r="E27" s="12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F27" s="13" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G27" s="41" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I27" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J27" s="29">
         <v>1</v>
       </c>
       <c r="K27" s="25" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L27" s="28" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M27" s="3"/>
     </row>
@@ -1909,7 +1909,7 @@
         <v>4</v>
       </c>
       <c r="B28" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C28" s="24">
         <v>19</v>
@@ -1918,28 +1918,28 @@
         <v>18</v>
       </c>
       <c r="E28" s="12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F28" s="13" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G28" s="41" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H28" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I28" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J28" s="29">
         <v>3</v>
       </c>
       <c r="K28" s="25" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L28" s="28" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M28" s="3"/>
     </row>
@@ -1948,7 +1948,7 @@
         <v>6</v>
       </c>
       <c r="B29" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C29" s="24">
         <v>19</v>
@@ -1957,28 +1957,28 @@
         <v>18</v>
       </c>
       <c r="E29" s="12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F29" s="25" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G29" s="41" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H29" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I29" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J29" s="29">
         <v>3</v>
       </c>
       <c r="K29" s="13" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L29" s="28" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M29" s="3"/>
     </row>
@@ -1987,7 +1987,7 @@
         <v>7</v>
       </c>
       <c r="B30" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C30" s="24">
         <v>11</v>
@@ -1996,42 +1996,42 @@
         <v>17</v>
       </c>
       <c r="E30" s="12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F30" s="13" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G30" s="41" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="H30" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I30" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="J30" s="29">
         <v>0</v>
       </c>
       <c r="K30" s="25" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L30" s="28" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M30" s="26" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="N30" s="30" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="31" spans="1:17" ht="20" customHeight="1">
       <c r="A31" s="35" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="B31" s="35" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C31" s="44">
         <v>1</v>
@@ -2040,32 +2040,32 @@
         <v>16</v>
       </c>
       <c r="E31" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="F31" s="45" t="s">
+        <v>17</v>
+      </c>
+      <c r="G31" s="41" t="s">
+        <v>24</v>
+      </c>
+      <c r="H31" s="43" t="s">
         <v>18</v>
       </c>
-      <c r="F31" s="45" t="s">
+      <c r="I31" s="43" t="s">
         <v>18</v>
       </c>
-      <c r="G31" s="41" t="s">
-        <v>25</v>
-      </c>
-      <c r="H31" s="43" t="s">
-        <v>19</v>
-      </c>
-      <c r="I31" s="43" t="s">
-        <v>19</v>
-      </c>
       <c r="J31" s="43" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K31" s="45" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="L31" s="46" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="M31" s="43"/>
       <c r="N31" s="35" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="32" spans="1:17" ht="20" customHeight="1">
@@ -2073,7 +2073,7 @@
         <v>3</v>
       </c>
       <c r="B32" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C32" s="21">
         <v>11</v>
@@ -2082,37 +2082,37 @@
         <v>11</v>
       </c>
       <c r="E32" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="F32" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="G32" s="41" t="s">
+        <v>17</v>
+      </c>
+      <c r="H32" s="3" t="s">
+        <v>17</v>
+      </c>
+      <c r="I32" s="3" t="s">
         <v>18</v>
-      </c>
-      <c r="F32" s="13" t="s">
-        <v>18</v>
-      </c>
-      <c r="G32" s="41" t="s">
-        <v>18</v>
-      </c>
-      <c r="H32" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="I32" s="3" t="s">
-        <v>19</v>
       </c>
       <c r="J32" s="29">
         <v>0</v>
       </c>
       <c r="K32" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="L32" s="28" t="s">
         <v>18</v>
-      </c>
-      <c r="L32" s="28" t="s">
-        <v>19</v>
       </c>
       <c r="M32" s="3"/>
     </row>
     <row r="33" spans="1:14" ht="20" customHeight="1">
       <c r="A33" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="B33" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C33" s="21">
         <v>10</v>
@@ -2121,39 +2121,39 @@
         <v>10</v>
       </c>
       <c r="E33" s="12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F33" s="23" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="G33" s="41" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H33" s="3" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="I33" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="J33" s="3">
         <v>6</v>
       </c>
       <c r="K33" s="13" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="L33" s="28" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="M33" s="26" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="34" spans="1:14" ht="20" customHeight="1">
       <c r="A34" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="B34" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C34" s="24">
         <v>1</v>
@@ -2162,37 +2162,37 @@
         <v>1</v>
       </c>
       <c r="E34" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="F34" s="23" t="s">
+        <v>54</v>
+      </c>
+      <c r="G34" s="41" t="s">
+        <v>24</v>
+      </c>
+      <c r="H34" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="F34" s="23" t="s">
-        <v>55</v>
-      </c>
-      <c r="G34" s="41" t="s">
-        <v>25</v>
-      </c>
-      <c r="H34" s="3" t="s">
-        <v>19</v>
-      </c>
       <c r="I34" s="3" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="J34" s="26" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K34" s="25" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="L34" s="27" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="M34" s="3"/>
     </row>
     <row r="35" spans="1:14" ht="20" customHeight="1">
       <c r="A35" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="B35" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C35" s="24">
         <v>1</v>
@@ -2201,37 +2201,37 @@
         <v>14</v>
       </c>
       <c r="E35" s="12" t="s">
+        <v>17</v>
+      </c>
+      <c r="F35" s="13" t="s">
+        <v>17</v>
+      </c>
+      <c r="G35" s="41" t="s">
+        <v>24</v>
+      </c>
+      <c r="H35" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="F35" s="13" t="s">
+      <c r="I35" s="3" t="s">
         <v>18</v>
       </c>
-      <c r="G35" s="41" t="s">
-        <v>25</v>
-      </c>
-      <c r="H35" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="I35" s="3" t="s">
-        <v>19</v>
-      </c>
       <c r="J35" s="26" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="K35" s="25" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="L35" s="27" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="M35" s="3"/>
       <c r="N35" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="36" spans="1:14" ht="20" customHeight="1">
       <c r="A36" s="4" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B36" s="4" t="s">
         <v>8</v>
@@ -2243,36 +2243,36 @@
         <v>2</v>
       </c>
       <c r="E36" s="12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F36" s="23" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="G36" s="41" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H36" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I36" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="J36" s="5" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="K36" s="23" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="L36" s="28" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M36" s="26" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="37" spans="1:14" ht="20" customHeight="1">
       <c r="A37" s="4" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B37" s="4" t="s">
         <v>8</v>
@@ -2284,31 +2284,31 @@
         <v>2</v>
       </c>
       <c r="E37" s="12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="F37" s="13" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="G37" s="41" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H37" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="I37" s="3" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="J37" s="3">
         <v>1</v>
       </c>
       <c r="K37" s="25" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="L37" s="28" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="M37" s="26" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
     </row>
     <row r="38" spans="1:14" ht="20" customHeight="1" thickBot="1">
@@ -2326,11 +2326,11 @@
     </row>
     <row r="39" spans="1:14" ht="18" thickTop="1" thickBot="1">
       <c r="A39" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C39" s="9">
         <f>SUM(C23:C37)</f>
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="D39" s="9">
         <f>SUM(D23:D37)</f>
@@ -2348,11 +2348,11 @@
     </row>
     <row r="40" spans="1:14" ht="18" thickTop="1" thickBot="1">
       <c r="A40" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C40" s="40">
         <f>1 - C39/D39</f>
-        <v>0.27572016460905346</v>
+        <v>0.27160493827160492</v>
       </c>
     </row>
     <row r="41" spans="1:14" ht="17" thickTop="1">
@@ -2363,36 +2363,36 @@
     </row>
     <row r="42" spans="1:14">
       <c r="A42" t="s">
+        <v>59</v>
+      </c>
+      <c r="B42" t="s">
+        <v>61</v>
+      </c>
+      <c r="C42" s="3" t="s">
+        <v>23</v>
+      </c>
+      <c r="D42" s="31" t="s">
+        <v>58</v>
+      </c>
+      <c r="E42" s="3" t="s">
+        <v>64</v>
+      </c>
+      <c r="F42" s="3" t="s">
+        <v>65</v>
+      </c>
+      <c r="G42" s="3" t="s">
+        <v>67</v>
+      </c>
+      <c r="H42" s="2" t="s">
         <v>60</v>
       </c>
-      <c r="B42" t="s">
-        <v>62</v>
-      </c>
-      <c r="C42" s="3" t="s">
-        <v>24</v>
-      </c>
-      <c r="D42" s="31" t="s">
-        <v>59</v>
-      </c>
-      <c r="E42" s="3" t="s">
-        <v>65</v>
-      </c>
-      <c r="F42" s="3" t="s">
-        <v>66</v>
-      </c>
-      <c r="G42" s="3" t="s">
-        <v>68</v>
-      </c>
-      <c r="H42" s="2" t="s">
-        <v>61</v>
-      </c>
       <c r="I42" s="3" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="43" spans="1:14" ht="20" customHeight="1">
       <c r="A43" s="4" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B43" s="4" t="s">
         <v>8</v>
@@ -2411,19 +2411,19 @@
         <v>2</v>
       </c>
       <c r="G43" s="33" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="H43" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I43" s="3"/>
     </row>
     <row r="44" spans="1:14" ht="20" customHeight="1">
       <c r="A44" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="B44" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C44" s="5">
         <v>0</v>
@@ -2436,18 +2436,18 @@
         <v>31</v>
       </c>
       <c r="F44" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="G44" s="3" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="45" spans="1:14" ht="20" customHeight="1">
       <c r="A45" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="B45" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C45" s="3">
         <v>78</v>
@@ -2467,16 +2467,16 @@
         <v>0.36708860759493672</v>
       </c>
       <c r="H45" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I45" s="3"/>
     </row>
     <row r="46" spans="1:14" ht="20" customHeight="1">
       <c r="A46" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B46" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C46" s="3">
         <v>10</v>
@@ -2496,10 +2496,10 @@
         <v>0.6</v>
       </c>
       <c r="H46" s="3" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="I46" s="31" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="47" spans="1:14" ht="17" thickBot="1">
@@ -2512,7 +2512,7 @@
     </row>
     <row r="48" spans="1:14" ht="18" thickTop="1" thickBot="1">
       <c r="A48" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="C48" s="9">
         <f>SUM(C44:C46)</f>
@@ -2533,14 +2533,14 @@
     </row>
     <row r="49" spans="1:9" ht="18" thickTop="1" thickBot="1">
       <c r="A49" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C49" s="40">
         <f>1 - C48/D48</f>
         <v>0.26666666666666672</v>
       </c>
       <c r="I49" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="50" spans="1:9" ht="17" thickTop="1"/>

</xml_diff>